<commit_message>
Regenerate all project outputs, reports, and dashboards with official MR logo branding and new validation engines
</commit_message>
<xml_diff>
--- a/analysis/Dapagliflozin/DAPA_HF_Trial_extracted.xlsx
+++ b/analysis/Dapagliflozin/DAPA_HF_Trial_extracted.xlsx
@@ -94,7 +94,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -116,11 +116,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -148,6 +192,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -222,6 +268,276 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>278</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>25</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>17</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>62</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -801,294 +1117,294 @@
           <t>STUDY &amp; INTERVENTION ARMS</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="12" t="n"/>
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ELIGIBILITY CRITERIA</t>
         </is>
       </c>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
-      <c r="AA1" s="1" t="n"/>
-      <c r="AB1" s="1" t="n"/>
-      <c r="AC1" s="1" t="n"/>
-      <c r="AD1" s="1" t="n"/>
-      <c r="AE1" s="1" t="n"/>
-      <c r="AF1" s="1" t="n"/>
-      <c r="AG1" s="1" t="n"/>
-      <c r="AH1" s="1" t="n"/>
-      <c r="AI1" s="1" t="n"/>
-      <c r="AJ1" s="1" t="n"/>
-      <c r="AK1" s="1" t="n"/>
-      <c r="AL1" s="1" t="n"/>
-      <c r="AM1" s="1" t="n"/>
-      <c r="AN1" s="1" t="n"/>
-      <c r="AO1" s="1" t="n"/>
-      <c r="AP1" s="1" t="n"/>
-      <c r="AQ1" s="1" t="n"/>
-      <c r="AR1" s="1" t="n"/>
-      <c r="AS1" s="1" t="n"/>
-      <c r="AT1" s="1" t="n"/>
-      <c r="AU1" s="1" t="n"/>
-      <c r="AV1" s="1" t="n"/>
-      <c r="AW1" s="1" t="n"/>
-      <c r="AX1" s="1" t="n"/>
-      <c r="AY1" s="1" t="n"/>
-      <c r="AZ1" s="1" t="n"/>
-      <c r="BA1" s="1" t="n"/>
+      <c r="L1" s="11" t="n"/>
+      <c r="M1" s="11" t="n"/>
+      <c r="N1" s="11" t="n"/>
+      <c r="O1" s="11" t="n"/>
+      <c r="P1" s="11" t="n"/>
+      <c r="Q1" s="11" t="n"/>
+      <c r="R1" s="11" t="n"/>
+      <c r="S1" s="11" t="n"/>
+      <c r="T1" s="11" t="n"/>
+      <c r="U1" s="11" t="n"/>
+      <c r="V1" s="11" t="n"/>
+      <c r="W1" s="11" t="n"/>
+      <c r="X1" s="11" t="n"/>
+      <c r="Y1" s="11" t="n"/>
+      <c r="Z1" s="11" t="n"/>
+      <c r="AA1" s="11" t="n"/>
+      <c r="AB1" s="11" t="n"/>
+      <c r="AC1" s="11" t="n"/>
+      <c r="AD1" s="11" t="n"/>
+      <c r="AE1" s="11" t="n"/>
+      <c r="AF1" s="11" t="n"/>
+      <c r="AG1" s="11" t="n"/>
+      <c r="AH1" s="11" t="n"/>
+      <c r="AI1" s="11" t="n"/>
+      <c r="AJ1" s="11" t="n"/>
+      <c r="AK1" s="11" t="n"/>
+      <c r="AL1" s="11" t="n"/>
+      <c r="AM1" s="11" t="n"/>
+      <c r="AN1" s="11" t="n"/>
+      <c r="AO1" s="11" t="n"/>
+      <c r="AP1" s="11" t="n"/>
+      <c r="AQ1" s="11" t="n"/>
+      <c r="AR1" s="11" t="n"/>
+      <c r="AS1" s="11" t="n"/>
+      <c r="AT1" s="11" t="n"/>
+      <c r="AU1" s="11" t="n"/>
+      <c r="AV1" s="11" t="n"/>
+      <c r="AW1" s="11" t="n"/>
+      <c r="AX1" s="11" t="n"/>
+      <c r="AY1" s="11" t="n"/>
+      <c r="AZ1" s="11" t="n"/>
+      <c r="BA1" s="12" t="n"/>
       <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>POPULATION STRATIFICATION</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="n"/>
-      <c r="BD1" s="1" t="n"/>
-      <c r="BE1" s="1" t="n"/>
+      <c r="BC1" s="11" t="n"/>
+      <c r="BD1" s="11" t="n"/>
+      <c r="BE1" s="12" t="n"/>
       <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>CLINICAL VARIABLES &amp; OUTCOMES</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="n"/>
-      <c r="BH1" s="1" t="n"/>
-      <c r="BI1" s="1" t="n"/>
-      <c r="BJ1" s="1" t="n"/>
-      <c r="BK1" s="1" t="n"/>
-      <c r="BL1" s="1" t="n"/>
-      <c r="BM1" s="1" t="n"/>
-      <c r="BN1" s="1" t="n"/>
-      <c r="BO1" s="1" t="n"/>
-      <c r="BP1" s="1" t="n"/>
-      <c r="BQ1" s="1" t="n"/>
-      <c r="BR1" s="1" t="n"/>
-      <c r="BS1" s="1" t="n"/>
-      <c r="BT1" s="1" t="n"/>
-      <c r="BU1" s="1" t="n"/>
-      <c r="BV1" s="1" t="n"/>
-      <c r="BW1" s="1" t="n"/>
-      <c r="BX1" s="1" t="n"/>
-      <c r="BY1" s="1" t="n"/>
-      <c r="BZ1" s="1" t="n"/>
-      <c r="CA1" s="1" t="n"/>
-      <c r="CB1" s="1" t="n"/>
-      <c r="CC1" s="1" t="n"/>
-      <c r="CD1" s="1" t="n"/>
-      <c r="CE1" s="1" t="n"/>
-      <c r="CF1" s="1" t="n"/>
-      <c r="CG1" s="1" t="n"/>
-      <c r="CH1" s="1" t="n"/>
-      <c r="CI1" s="1" t="n"/>
-      <c r="CJ1" s="1" t="n"/>
-      <c r="CK1" s="1" t="n"/>
-      <c r="CL1" s="1" t="n"/>
-      <c r="CM1" s="1" t="n"/>
-      <c r="CN1" s="1" t="n"/>
-      <c r="CO1" s="1" t="n"/>
-      <c r="CP1" s="1" t="n"/>
-      <c r="CQ1" s="1" t="n"/>
-      <c r="CR1" s="1" t="n"/>
-      <c r="CS1" s="1" t="n"/>
-      <c r="CT1" s="1" t="n"/>
-      <c r="CU1" s="1" t="n"/>
-      <c r="CV1" s="1" t="n"/>
-      <c r="CW1" s="1" t="n"/>
-      <c r="CX1" s="1" t="n"/>
-      <c r="CY1" s="1" t="n"/>
-      <c r="CZ1" s="1" t="n"/>
-      <c r="DA1" s="1" t="n"/>
-      <c r="DB1" s="1" t="n"/>
-      <c r="DC1" s="1" t="n"/>
-      <c r="DD1" s="1" t="n"/>
-      <c r="DE1" s="1" t="n"/>
-      <c r="DF1" s="1" t="n"/>
-      <c r="DG1" s="1" t="n"/>
-      <c r="DH1" s="1" t="n"/>
-      <c r="DI1" s="1" t="n"/>
-      <c r="DJ1" s="1" t="n"/>
-      <c r="DK1" s="1" t="n"/>
-      <c r="DL1" s="1" t="n"/>
-      <c r="DM1" s="1" t="n"/>
-      <c r="DN1" s="1" t="n"/>
-      <c r="DO1" s="1" t="n"/>
-      <c r="DP1" s="1" t="n"/>
-      <c r="DQ1" s="1" t="n"/>
-      <c r="DR1" s="1" t="n"/>
-      <c r="DS1" s="1" t="n"/>
-      <c r="DT1" s="1" t="n"/>
-      <c r="DU1" s="1" t="n"/>
-      <c r="DV1" s="1" t="n"/>
-      <c r="DW1" s="1" t="n"/>
-      <c r="DX1" s="1" t="n"/>
-      <c r="DY1" s="1" t="n"/>
-      <c r="DZ1" s="1" t="n"/>
-      <c r="EA1" s="1" t="n"/>
-      <c r="EB1" s="1" t="n"/>
-      <c r="EC1" s="1" t="n"/>
-      <c r="ED1" s="1" t="n"/>
-      <c r="EE1" s="1" t="n"/>
-      <c r="EF1" s="1" t="n"/>
-      <c r="EG1" s="1" t="n"/>
-      <c r="EH1" s="1" t="n"/>
-      <c r="EI1" s="1" t="n"/>
-      <c r="EJ1" s="1" t="n"/>
-      <c r="EK1" s="1" t="n"/>
-      <c r="EL1" s="1" t="n"/>
-      <c r="EM1" s="1" t="n"/>
-      <c r="EN1" s="1" t="n"/>
-      <c r="EO1" s="1" t="n"/>
-      <c r="EP1" s="1" t="n"/>
-      <c r="EQ1" s="1" t="n"/>
-      <c r="ER1" s="1" t="n"/>
-      <c r="ES1" s="1" t="n"/>
-      <c r="ET1" s="1" t="n"/>
-      <c r="EU1" s="1" t="n"/>
-      <c r="EV1" s="1" t="n"/>
-      <c r="EW1" s="1" t="n"/>
-      <c r="EX1" s="1" t="n"/>
-      <c r="EY1" s="1" t="n"/>
-      <c r="EZ1" s="1" t="n"/>
-      <c r="FA1" s="1" t="n"/>
-      <c r="FB1" s="1" t="n"/>
-      <c r="FC1" s="1" t="n"/>
-      <c r="FD1" s="1" t="n"/>
-      <c r="FE1" s="1" t="n"/>
-      <c r="FF1" s="1" t="n"/>
-      <c r="FG1" s="1" t="n"/>
-      <c r="FH1" s="1" t="n"/>
-      <c r="FI1" s="1" t="n"/>
-      <c r="FJ1" s="1" t="n"/>
-      <c r="FK1" s="1" t="n"/>
-      <c r="FL1" s="1" t="n"/>
-      <c r="FM1" s="1" t="n"/>
-      <c r="FN1" s="1" t="n"/>
-      <c r="FO1" s="1" t="n"/>
-      <c r="FP1" s="1" t="n"/>
-      <c r="FQ1" s="1" t="n"/>
-      <c r="FR1" s="1" t="n"/>
-      <c r="FS1" s="1" t="n"/>
-      <c r="FT1" s="1" t="n"/>
-      <c r="FU1" s="1" t="n"/>
-      <c r="FV1" s="1" t="n"/>
-      <c r="FW1" s="1" t="n"/>
-      <c r="FX1" s="1" t="n"/>
-      <c r="FY1" s="1" t="n"/>
-      <c r="FZ1" s="1" t="n"/>
-      <c r="GA1" s="1" t="n"/>
-      <c r="GB1" s="1" t="n"/>
-      <c r="GC1" s="1" t="n"/>
-      <c r="GD1" s="1" t="n"/>
-      <c r="GE1" s="1" t="n"/>
-      <c r="GF1" s="1" t="n"/>
-      <c r="GG1" s="1" t="n"/>
-      <c r="GH1" s="1" t="n"/>
-      <c r="GI1" s="1" t="n"/>
-      <c r="GJ1" s="1" t="n"/>
-      <c r="GK1" s="1" t="n"/>
-      <c r="GL1" s="1" t="n"/>
-      <c r="GM1" s="1" t="n"/>
-      <c r="GN1" s="1" t="n"/>
-      <c r="GO1" s="1" t="n"/>
-      <c r="GP1" s="1" t="n"/>
-      <c r="GQ1" s="1" t="n"/>
-      <c r="GR1" s="1" t="n"/>
-      <c r="GS1" s="1" t="n"/>
-      <c r="GT1" s="1" t="n"/>
-      <c r="GU1" s="1" t="n"/>
-      <c r="GV1" s="1" t="n"/>
-      <c r="GW1" s="1" t="n"/>
-      <c r="GX1" s="1" t="n"/>
-      <c r="GY1" s="1" t="n"/>
-      <c r="GZ1" s="1" t="n"/>
-      <c r="HA1" s="1" t="n"/>
-      <c r="HB1" s="1" t="n"/>
-      <c r="HC1" s="1" t="n"/>
-      <c r="HD1" s="1" t="n"/>
-      <c r="HE1" s="1" t="n"/>
-      <c r="HF1" s="1" t="n"/>
-      <c r="HG1" s="1" t="n"/>
-      <c r="HH1" s="1" t="n"/>
-      <c r="HI1" s="1" t="n"/>
-      <c r="HJ1" s="1" t="n"/>
-      <c r="HK1" s="1" t="n"/>
-      <c r="HL1" s="1" t="n"/>
-      <c r="HM1" s="1" t="n"/>
-      <c r="HN1" s="1" t="n"/>
-      <c r="HO1" s="1" t="n"/>
-      <c r="HP1" s="1" t="n"/>
-      <c r="HQ1" s="1" t="n"/>
-      <c r="HR1" s="1" t="n"/>
-      <c r="HS1" s="1" t="n"/>
-      <c r="HT1" s="1" t="n"/>
-      <c r="HU1" s="1" t="n"/>
-      <c r="HV1" s="1" t="n"/>
-      <c r="HW1" s="1" t="n"/>
-      <c r="HX1" s="1" t="n"/>
-      <c r="HY1" s="1" t="n"/>
-      <c r="HZ1" s="1" t="n"/>
-      <c r="IA1" s="1" t="n"/>
-      <c r="IB1" s="1" t="n"/>
-      <c r="IC1" s="1" t="n"/>
-      <c r="ID1" s="1" t="n"/>
-      <c r="IE1" s="1" t="n"/>
-      <c r="IF1" s="1" t="n"/>
-      <c r="IG1" s="1" t="n"/>
-      <c r="IH1" s="1" t="n"/>
-      <c r="II1" s="1" t="n"/>
-      <c r="IJ1" s="1" t="n"/>
-      <c r="IK1" s="1" t="n"/>
-      <c r="IL1" s="1" t="n"/>
-      <c r="IM1" s="1" t="n"/>
-      <c r="IN1" s="1" t="n"/>
-      <c r="IO1" s="1" t="n"/>
-      <c r="IP1" s="1" t="n"/>
-      <c r="IQ1" s="1" t="n"/>
-      <c r="IR1" s="1" t="n"/>
-      <c r="IS1" s="1" t="n"/>
-      <c r="IT1" s="1" t="n"/>
-      <c r="IU1" s="1" t="n"/>
-      <c r="IV1" s="1" t="n"/>
-      <c r="IW1" s="1" t="n"/>
-      <c r="IX1" s="1" t="n"/>
-      <c r="IY1" s="1" t="n"/>
-      <c r="IZ1" s="1" t="n"/>
-      <c r="JA1" s="1" t="n"/>
-      <c r="JB1" s="1" t="n"/>
-      <c r="JC1" s="1" t="n"/>
-      <c r="JD1" s="1" t="n"/>
-      <c r="JE1" s="1" t="n"/>
-      <c r="JF1" s="1" t="n"/>
-      <c r="JG1" s="1" t="n"/>
-      <c r="JH1" s="1" t="n"/>
-      <c r="JI1" s="1" t="n"/>
-      <c r="JJ1" s="1" t="n"/>
-      <c r="JK1" s="1" t="n"/>
-      <c r="JL1" s="1" t="n"/>
-      <c r="JM1" s="1" t="n"/>
-      <c r="JN1" s="1" t="n"/>
-      <c r="JO1" s="1" t="n"/>
-      <c r="JP1" s="1" t="n"/>
-      <c r="JQ1" s="1" t="n"/>
+      <c r="BG1" s="11" t="n"/>
+      <c r="BH1" s="11" t="n"/>
+      <c r="BI1" s="11" t="n"/>
+      <c r="BJ1" s="11" t="n"/>
+      <c r="BK1" s="11" t="n"/>
+      <c r="BL1" s="11" t="n"/>
+      <c r="BM1" s="11" t="n"/>
+      <c r="BN1" s="11" t="n"/>
+      <c r="BO1" s="11" t="n"/>
+      <c r="BP1" s="11" t="n"/>
+      <c r="BQ1" s="11" t="n"/>
+      <c r="BR1" s="11" t="n"/>
+      <c r="BS1" s="11" t="n"/>
+      <c r="BT1" s="11" t="n"/>
+      <c r="BU1" s="11" t="n"/>
+      <c r="BV1" s="11" t="n"/>
+      <c r="BW1" s="11" t="n"/>
+      <c r="BX1" s="11" t="n"/>
+      <c r="BY1" s="11" t="n"/>
+      <c r="BZ1" s="11" t="n"/>
+      <c r="CA1" s="11" t="n"/>
+      <c r="CB1" s="11" t="n"/>
+      <c r="CC1" s="11" t="n"/>
+      <c r="CD1" s="11" t="n"/>
+      <c r="CE1" s="11" t="n"/>
+      <c r="CF1" s="11" t="n"/>
+      <c r="CG1" s="11" t="n"/>
+      <c r="CH1" s="11" t="n"/>
+      <c r="CI1" s="11" t="n"/>
+      <c r="CJ1" s="11" t="n"/>
+      <c r="CK1" s="11" t="n"/>
+      <c r="CL1" s="11" t="n"/>
+      <c r="CM1" s="11" t="n"/>
+      <c r="CN1" s="11" t="n"/>
+      <c r="CO1" s="11" t="n"/>
+      <c r="CP1" s="11" t="n"/>
+      <c r="CQ1" s="11" t="n"/>
+      <c r="CR1" s="11" t="n"/>
+      <c r="CS1" s="11" t="n"/>
+      <c r="CT1" s="11" t="n"/>
+      <c r="CU1" s="11" t="n"/>
+      <c r="CV1" s="11" t="n"/>
+      <c r="CW1" s="11" t="n"/>
+      <c r="CX1" s="11" t="n"/>
+      <c r="CY1" s="11" t="n"/>
+      <c r="CZ1" s="11" t="n"/>
+      <c r="DA1" s="11" t="n"/>
+      <c r="DB1" s="11" t="n"/>
+      <c r="DC1" s="11" t="n"/>
+      <c r="DD1" s="11" t="n"/>
+      <c r="DE1" s="11" t="n"/>
+      <c r="DF1" s="11" t="n"/>
+      <c r="DG1" s="11" t="n"/>
+      <c r="DH1" s="11" t="n"/>
+      <c r="DI1" s="11" t="n"/>
+      <c r="DJ1" s="11" t="n"/>
+      <c r="DK1" s="11" t="n"/>
+      <c r="DL1" s="11" t="n"/>
+      <c r="DM1" s="11" t="n"/>
+      <c r="DN1" s="11" t="n"/>
+      <c r="DO1" s="11" t="n"/>
+      <c r="DP1" s="11" t="n"/>
+      <c r="DQ1" s="11" t="n"/>
+      <c r="DR1" s="11" t="n"/>
+      <c r="DS1" s="11" t="n"/>
+      <c r="DT1" s="11" t="n"/>
+      <c r="DU1" s="11" t="n"/>
+      <c r="DV1" s="11" t="n"/>
+      <c r="DW1" s="11" t="n"/>
+      <c r="DX1" s="11" t="n"/>
+      <c r="DY1" s="11" t="n"/>
+      <c r="DZ1" s="11" t="n"/>
+      <c r="EA1" s="11" t="n"/>
+      <c r="EB1" s="11" t="n"/>
+      <c r="EC1" s="11" t="n"/>
+      <c r="ED1" s="11" t="n"/>
+      <c r="EE1" s="11" t="n"/>
+      <c r="EF1" s="11" t="n"/>
+      <c r="EG1" s="11" t="n"/>
+      <c r="EH1" s="11" t="n"/>
+      <c r="EI1" s="11" t="n"/>
+      <c r="EJ1" s="11" t="n"/>
+      <c r="EK1" s="11" t="n"/>
+      <c r="EL1" s="11" t="n"/>
+      <c r="EM1" s="11" t="n"/>
+      <c r="EN1" s="11" t="n"/>
+      <c r="EO1" s="11" t="n"/>
+      <c r="EP1" s="11" t="n"/>
+      <c r="EQ1" s="11" t="n"/>
+      <c r="ER1" s="11" t="n"/>
+      <c r="ES1" s="11" t="n"/>
+      <c r="ET1" s="11" t="n"/>
+      <c r="EU1" s="11" t="n"/>
+      <c r="EV1" s="11" t="n"/>
+      <c r="EW1" s="11" t="n"/>
+      <c r="EX1" s="11" t="n"/>
+      <c r="EY1" s="11" t="n"/>
+      <c r="EZ1" s="11" t="n"/>
+      <c r="FA1" s="11" t="n"/>
+      <c r="FB1" s="11" t="n"/>
+      <c r="FC1" s="11" t="n"/>
+      <c r="FD1" s="11" t="n"/>
+      <c r="FE1" s="11" t="n"/>
+      <c r="FF1" s="11" t="n"/>
+      <c r="FG1" s="11" t="n"/>
+      <c r="FH1" s="11" t="n"/>
+      <c r="FI1" s="11" t="n"/>
+      <c r="FJ1" s="11" t="n"/>
+      <c r="FK1" s="11" t="n"/>
+      <c r="FL1" s="11" t="n"/>
+      <c r="FM1" s="11" t="n"/>
+      <c r="FN1" s="11" t="n"/>
+      <c r="FO1" s="11" t="n"/>
+      <c r="FP1" s="11" t="n"/>
+      <c r="FQ1" s="11" t="n"/>
+      <c r="FR1" s="11" t="n"/>
+      <c r="FS1" s="11" t="n"/>
+      <c r="FT1" s="11" t="n"/>
+      <c r="FU1" s="11" t="n"/>
+      <c r="FV1" s="11" t="n"/>
+      <c r="FW1" s="11" t="n"/>
+      <c r="FX1" s="11" t="n"/>
+      <c r="FY1" s="11" t="n"/>
+      <c r="FZ1" s="11" t="n"/>
+      <c r="GA1" s="11" t="n"/>
+      <c r="GB1" s="11" t="n"/>
+      <c r="GC1" s="11" t="n"/>
+      <c r="GD1" s="11" t="n"/>
+      <c r="GE1" s="11" t="n"/>
+      <c r="GF1" s="11" t="n"/>
+      <c r="GG1" s="11" t="n"/>
+      <c r="GH1" s="11" t="n"/>
+      <c r="GI1" s="11" t="n"/>
+      <c r="GJ1" s="11" t="n"/>
+      <c r="GK1" s="11" t="n"/>
+      <c r="GL1" s="11" t="n"/>
+      <c r="GM1" s="11" t="n"/>
+      <c r="GN1" s="11" t="n"/>
+      <c r="GO1" s="11" t="n"/>
+      <c r="GP1" s="11" t="n"/>
+      <c r="GQ1" s="11" t="n"/>
+      <c r="GR1" s="11" t="n"/>
+      <c r="GS1" s="11" t="n"/>
+      <c r="GT1" s="11" t="n"/>
+      <c r="GU1" s="11" t="n"/>
+      <c r="GV1" s="11" t="n"/>
+      <c r="GW1" s="11" t="n"/>
+      <c r="GX1" s="11" t="n"/>
+      <c r="GY1" s="11" t="n"/>
+      <c r="GZ1" s="11" t="n"/>
+      <c r="HA1" s="11" t="n"/>
+      <c r="HB1" s="11" t="n"/>
+      <c r="HC1" s="11" t="n"/>
+      <c r="HD1" s="11" t="n"/>
+      <c r="HE1" s="11" t="n"/>
+      <c r="HF1" s="11" t="n"/>
+      <c r="HG1" s="11" t="n"/>
+      <c r="HH1" s="11" t="n"/>
+      <c r="HI1" s="11" t="n"/>
+      <c r="HJ1" s="11" t="n"/>
+      <c r="HK1" s="11" t="n"/>
+      <c r="HL1" s="11" t="n"/>
+      <c r="HM1" s="11" t="n"/>
+      <c r="HN1" s="11" t="n"/>
+      <c r="HO1" s="11" t="n"/>
+      <c r="HP1" s="11" t="n"/>
+      <c r="HQ1" s="11" t="n"/>
+      <c r="HR1" s="11" t="n"/>
+      <c r="HS1" s="11" t="n"/>
+      <c r="HT1" s="11" t="n"/>
+      <c r="HU1" s="11" t="n"/>
+      <c r="HV1" s="11" t="n"/>
+      <c r="HW1" s="11" t="n"/>
+      <c r="HX1" s="11" t="n"/>
+      <c r="HY1" s="11" t="n"/>
+      <c r="HZ1" s="11" t="n"/>
+      <c r="IA1" s="11" t="n"/>
+      <c r="IB1" s="11" t="n"/>
+      <c r="IC1" s="11" t="n"/>
+      <c r="ID1" s="11" t="n"/>
+      <c r="IE1" s="11" t="n"/>
+      <c r="IF1" s="11" t="n"/>
+      <c r="IG1" s="11" t="n"/>
+      <c r="IH1" s="11" t="n"/>
+      <c r="II1" s="11" t="n"/>
+      <c r="IJ1" s="11" t="n"/>
+      <c r="IK1" s="11" t="n"/>
+      <c r="IL1" s="11" t="n"/>
+      <c r="IM1" s="11" t="n"/>
+      <c r="IN1" s="11" t="n"/>
+      <c r="IO1" s="11" t="n"/>
+      <c r="IP1" s="11" t="n"/>
+      <c r="IQ1" s="11" t="n"/>
+      <c r="IR1" s="11" t="n"/>
+      <c r="IS1" s="11" t="n"/>
+      <c r="IT1" s="11" t="n"/>
+      <c r="IU1" s="11" t="n"/>
+      <c r="IV1" s="11" t="n"/>
+      <c r="IW1" s="11" t="n"/>
+      <c r="IX1" s="11" t="n"/>
+      <c r="IY1" s="11" t="n"/>
+      <c r="IZ1" s="11" t="n"/>
+      <c r="JA1" s="11" t="n"/>
+      <c r="JB1" s="11" t="n"/>
+      <c r="JC1" s="11" t="n"/>
+      <c r="JD1" s="11" t="n"/>
+      <c r="JE1" s="11" t="n"/>
+      <c r="JF1" s="11" t="n"/>
+      <c r="JG1" s="11" t="n"/>
+      <c r="JH1" s="11" t="n"/>
+      <c r="JI1" s="11" t="n"/>
+      <c r="JJ1" s="11" t="n"/>
+      <c r="JK1" s="11" t="n"/>
+      <c r="JL1" s="11" t="n"/>
+      <c r="JM1" s="11" t="n"/>
+      <c r="JN1" s="11" t="n"/>
+      <c r="JO1" s="11" t="n"/>
+      <c r="JP1" s="11" t="n"/>
+      <c r="JQ1" s="12" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1126,7 +1442,7 @@
           <t>Period of Study</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n"/>
+      <c r="H2" s="12" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Total Cohort (N)</t>
@@ -1142,64 +1458,64 @@
           <t>Age</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
+      <c r="L2" s="11" t="n"/>
+      <c r="M2" s="11" t="n"/>
+      <c r="N2" s="11" t="n"/>
+      <c r="O2" s="12" t="n"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Ejection Fraction</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
+      <c r="Q2" s="11" t="n"/>
+      <c r="R2" s="11" t="n"/>
+      <c r="S2" s="11" t="n"/>
+      <c r="T2" s="12" t="n"/>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Nyha Class</t>
         </is>
       </c>
-      <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="n"/>
-      <c r="X2" s="2" t="n"/>
-      <c r="Y2" s="2" t="n"/>
+      <c r="V2" s="11" t="n"/>
+      <c r="W2" s="11" t="n"/>
+      <c r="X2" s="11" t="n"/>
+      <c r="Y2" s="12" t="n"/>
       <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Nt Probnp</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="n"/>
-      <c r="AB2" s="2" t="n"/>
-      <c r="AC2" s="2" t="n"/>
-      <c r="AD2" s="2" t="n"/>
+      <c r="AA2" s="11" t="n"/>
+      <c r="AB2" s="11" t="n"/>
+      <c r="AC2" s="11" t="n"/>
+      <c r="AD2" s="12" t="n"/>
       <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>Nt Probnp Afib</t>
         </is>
       </c>
-      <c r="AF2" s="2" t="n"/>
-      <c r="AG2" s="2" t="n"/>
-      <c r="AH2" s="2" t="n"/>
-      <c r="AI2" s="2" t="n"/>
+      <c r="AF2" s="11" t="n"/>
+      <c r="AG2" s="11" t="n"/>
+      <c r="AH2" s="11" t="n"/>
+      <c r="AI2" s="12" t="n"/>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>Systolic Blood Pressure</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="n"/>
-      <c r="AL2" s="2" t="n"/>
-      <c r="AM2" s="2" t="n"/>
-      <c r="AN2" s="2" t="n"/>
+      <c r="AK2" s="11" t="n"/>
+      <c r="AL2" s="11" t="n"/>
+      <c r="AM2" s="11" t="n"/>
+      <c r="AN2" s="12" t="n"/>
       <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>Egfr</t>
         </is>
       </c>
-      <c r="AP2" s="2" t="n"/>
-      <c r="AQ2" s="2" t="n"/>
-      <c r="AR2" s="2" t="n"/>
-      <c r="AS2" s="2" t="n"/>
+      <c r="AP2" s="11" t="n"/>
+      <c r="AQ2" s="11" t="n"/>
+      <c r="AR2" s="11" t="n"/>
+      <c r="AS2" s="12" t="n"/>
       <c r="AT2" s="2" t="inlineStr">
         <is>
           <t>Standard Hf Therapy</t>
@@ -1255,447 +1571,447 @@
           <t>Timepoint</t>
         </is>
       </c>
-      <c r="BE2" s="2" t="n"/>
+      <c r="BE2" s="12" t="n"/>
       <c r="BF2" s="2" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="BG2" s="2" t="n"/>
-      <c r="BH2" s="2" t="n"/>
-      <c r="BI2" s="2" t="n"/>
+      <c r="BG2" s="11" t="n"/>
+      <c r="BH2" s="11" t="n"/>
+      <c r="BI2" s="12" t="n"/>
       <c r="BJ2" s="2" t="inlineStr">
         <is>
           <t>Female Sex</t>
         </is>
       </c>
-      <c r="BK2" s="2" t="n"/>
-      <c r="BL2" s="2" t="n"/>
-      <c r="BM2" s="2" t="n"/>
+      <c r="BK2" s="11" t="n"/>
+      <c r="BL2" s="11" t="n"/>
+      <c r="BM2" s="12" t="n"/>
       <c r="BN2" s="2" t="inlineStr">
         <is>
           <t>BMI</t>
         </is>
       </c>
-      <c r="BO2" s="2" t="n"/>
-      <c r="BP2" s="2" t="n"/>
-      <c r="BQ2" s="2" t="n"/>
+      <c r="BO2" s="11" t="n"/>
+      <c r="BP2" s="11" t="n"/>
+      <c r="BQ2" s="12" t="n"/>
       <c r="BR2" s="2" t="inlineStr">
         <is>
           <t>Race Distribution</t>
         </is>
       </c>
-      <c r="BS2" s="2" t="n"/>
-      <c r="BT2" s="2" t="n"/>
-      <c r="BU2" s="2" t="n"/>
+      <c r="BS2" s="11" t="n"/>
+      <c r="BT2" s="11" t="n"/>
+      <c r="BU2" s="12" t="n"/>
       <c r="BV2" s="2" t="inlineStr">
         <is>
           <t>Region - North America</t>
         </is>
       </c>
-      <c r="BW2" s="2" t="n"/>
-      <c r="BX2" s="2" t="n"/>
-      <c r="BY2" s="2" t="n"/>
+      <c r="BW2" s="11" t="n"/>
+      <c r="BX2" s="11" t="n"/>
+      <c r="BY2" s="12" t="n"/>
       <c r="BZ2" s="2" t="inlineStr">
         <is>
           <t>Region - South America</t>
         </is>
       </c>
-      <c r="CA2" s="2" t="n"/>
-      <c r="CB2" s="2" t="n"/>
-      <c r="CC2" s="2" t="n"/>
+      <c r="CA2" s="11" t="n"/>
+      <c r="CB2" s="11" t="n"/>
+      <c r="CC2" s="12" t="n"/>
       <c r="CD2" s="2" t="inlineStr">
         <is>
           <t>Region - Europe</t>
         </is>
       </c>
-      <c r="CE2" s="2" t="n"/>
-      <c r="CF2" s="2" t="n"/>
-      <c r="CG2" s="2" t="n"/>
+      <c r="CE2" s="11" t="n"/>
+      <c r="CF2" s="11" t="n"/>
+      <c r="CG2" s="12" t="n"/>
       <c r="CH2" s="2" t="inlineStr">
         <is>
           <t>Region - Asia–Pacific</t>
         </is>
       </c>
-      <c r="CI2" s="2" t="n"/>
-      <c r="CJ2" s="2" t="n"/>
-      <c r="CK2" s="2" t="n"/>
+      <c r="CI2" s="11" t="n"/>
+      <c r="CJ2" s="11" t="n"/>
+      <c r="CK2" s="12" t="n"/>
       <c r="CL2" s="2" t="inlineStr">
         <is>
           <t>NYHA Class II</t>
         </is>
       </c>
-      <c r="CM2" s="2" t="n"/>
-      <c r="CN2" s="2" t="n"/>
-      <c r="CO2" s="2" t="n"/>
+      <c r="CM2" s="11" t="n"/>
+      <c r="CN2" s="11" t="n"/>
+      <c r="CO2" s="12" t="n"/>
       <c r="CP2" s="2" t="inlineStr">
         <is>
           <t>NYHA Class III</t>
         </is>
       </c>
-      <c r="CQ2" s="2" t="n"/>
-      <c r="CR2" s="2" t="n"/>
-      <c r="CS2" s="2" t="n"/>
+      <c r="CQ2" s="11" t="n"/>
+      <c r="CR2" s="11" t="n"/>
+      <c r="CS2" s="12" t="n"/>
       <c r="CT2" s="2" t="inlineStr">
         <is>
           <t>NYHA Class IV</t>
         </is>
       </c>
-      <c r="CU2" s="2" t="n"/>
-      <c r="CV2" s="2" t="n"/>
-      <c r="CW2" s="2" t="n"/>
+      <c r="CU2" s="11" t="n"/>
+      <c r="CV2" s="11" t="n"/>
+      <c r="CW2" s="12" t="n"/>
       <c r="CX2" s="2" t="inlineStr">
         <is>
           <t>Heart Rate</t>
         </is>
       </c>
-      <c r="CY2" s="2" t="n"/>
-      <c r="CZ2" s="2" t="n"/>
-      <c r="DA2" s="2" t="n"/>
+      <c r="CY2" s="11" t="n"/>
+      <c r="CZ2" s="11" t="n"/>
+      <c r="DA2" s="12" t="n"/>
       <c r="DB2" s="2" t="inlineStr">
         <is>
           <t>Systolic Blood Pressure</t>
         </is>
       </c>
-      <c r="DC2" s="2" t="n"/>
-      <c r="DD2" s="2" t="n"/>
-      <c r="DE2" s="2" t="n"/>
+      <c r="DC2" s="11" t="n"/>
+      <c r="DD2" s="11" t="n"/>
+      <c r="DE2" s="12" t="n"/>
       <c r="DF2" s="2" t="inlineStr">
         <is>
           <t>Left Ventricular Ejection Fraction</t>
         </is>
       </c>
-      <c r="DG2" s="2" t="n"/>
-      <c r="DH2" s="2" t="n"/>
-      <c r="DI2" s="2" t="n"/>
+      <c r="DG2" s="11" t="n"/>
+      <c r="DH2" s="11" t="n"/>
+      <c r="DI2" s="12" t="n"/>
       <c r="DJ2" s="2" t="inlineStr">
         <is>
           <t>NT-proBNP</t>
         </is>
       </c>
-      <c r="DK2" s="2" t="n"/>
-      <c r="DL2" s="2" t="n"/>
-      <c r="DM2" s="2" t="n"/>
+      <c r="DK2" s="11" t="n"/>
+      <c r="DL2" s="11" t="n"/>
+      <c r="DM2" s="12" t="n"/>
       <c r="DN2" s="2" t="inlineStr">
         <is>
           <t>Cause of HF - Ischemic</t>
         </is>
       </c>
-      <c r="DO2" s="2" t="n"/>
-      <c r="DP2" s="2" t="n"/>
-      <c r="DQ2" s="2" t="n"/>
+      <c r="DO2" s="11" t="n"/>
+      <c r="DP2" s="11" t="n"/>
+      <c r="DQ2" s="12" t="n"/>
       <c r="DR2" s="2" t="inlineStr">
         <is>
           <t>Cause of HF - Nonischemic</t>
         </is>
       </c>
-      <c r="DS2" s="2" t="n"/>
-      <c r="DT2" s="2" t="n"/>
-      <c r="DU2" s="2" t="n"/>
+      <c r="DS2" s="11" t="n"/>
+      <c r="DT2" s="11" t="n"/>
+      <c r="DU2" s="12" t="n"/>
       <c r="DV2" s="2" t="inlineStr">
         <is>
           <t>Cause of HF - Unknown</t>
         </is>
       </c>
-      <c r="DW2" s="2" t="n"/>
-      <c r="DX2" s="2" t="n"/>
-      <c r="DY2" s="2" t="n"/>
+      <c r="DW2" s="11" t="n"/>
+      <c r="DX2" s="11" t="n"/>
+      <c r="DY2" s="12" t="n"/>
       <c r="DZ2" s="2" t="inlineStr">
         <is>
           <t>Hospitalization for Heart Failure</t>
         </is>
       </c>
-      <c r="EA2" s="2" t="n"/>
-      <c r="EB2" s="2" t="n"/>
-      <c r="EC2" s="2" t="n"/>
+      <c r="EA2" s="11" t="n"/>
+      <c r="EB2" s="11" t="n"/>
+      <c r="EC2" s="12" t="n"/>
       <c r="ED2" s="2" t="inlineStr">
         <is>
           <t>Atrial Fibrillation</t>
         </is>
       </c>
-      <c r="EE2" s="2" t="n"/>
-      <c r="EF2" s="2" t="n"/>
-      <c r="EG2" s="2" t="n"/>
+      <c r="EE2" s="11" t="n"/>
+      <c r="EF2" s="11" t="n"/>
+      <c r="EG2" s="12" t="n"/>
       <c r="EH2" s="2" t="inlineStr">
         <is>
           <t>Diabetes Mellitus</t>
         </is>
       </c>
-      <c r="EI2" s="2" t="n"/>
-      <c r="EJ2" s="2" t="n"/>
-      <c r="EK2" s="2" t="n"/>
+      <c r="EI2" s="11" t="n"/>
+      <c r="EJ2" s="11" t="n"/>
+      <c r="EK2" s="12" t="n"/>
       <c r="EL2" s="2" t="inlineStr">
         <is>
           <t>eGFR</t>
         </is>
       </c>
-      <c r="EM2" s="2" t="n"/>
-      <c r="EN2" s="2" t="n"/>
-      <c r="EO2" s="2" t="n"/>
+      <c r="EM2" s="11" t="n"/>
+      <c r="EN2" s="11" t="n"/>
+      <c r="EO2" s="12" t="n"/>
       <c r="EP2" s="2" t="inlineStr">
         <is>
           <t>eGFR &lt; 60 ml/min/1.73 m2</t>
         </is>
       </c>
-      <c r="EQ2" s="2" t="n"/>
-      <c r="ER2" s="2" t="n"/>
-      <c r="ES2" s="2" t="n"/>
+      <c r="EQ2" s="11" t="n"/>
+      <c r="ER2" s="11" t="n"/>
+      <c r="ES2" s="12" t="n"/>
       <c r="ET2" s="2" t="inlineStr">
         <is>
           <t>Device - Implantable Cardioverter–Defibrillator</t>
         </is>
       </c>
-      <c r="EU2" s="2" t="n"/>
-      <c r="EV2" s="2" t="n"/>
-      <c r="EW2" s="2" t="n"/>
+      <c r="EU2" s="11" t="n"/>
+      <c r="EV2" s="11" t="n"/>
+      <c r="EW2" s="12" t="n"/>
       <c r="EX2" s="2" t="inlineStr">
         <is>
           <t>Device - Cardiac Resynchronization Therapy</t>
         </is>
       </c>
-      <c r="EY2" s="2" t="n"/>
-      <c r="EZ2" s="2" t="n"/>
-      <c r="FA2" s="2" t="n"/>
+      <c r="EY2" s="11" t="n"/>
+      <c r="EZ2" s="11" t="n"/>
+      <c r="FA2" s="12" t="n"/>
       <c r="FB2" s="2" t="inlineStr">
         <is>
           <t>HF Med - Diuretic</t>
         </is>
       </c>
-      <c r="FC2" s="2" t="n"/>
-      <c r="FD2" s="2" t="n"/>
-      <c r="FE2" s="2" t="n"/>
+      <c r="FC2" s="11" t="n"/>
+      <c r="FD2" s="11" t="n"/>
+      <c r="FE2" s="12" t="n"/>
       <c r="FF2" s="2" t="inlineStr">
         <is>
           <t>HF Med - ACE Inhibitor</t>
         </is>
       </c>
-      <c r="FG2" s="2" t="n"/>
-      <c r="FH2" s="2" t="n"/>
-      <c r="FI2" s="2" t="n"/>
+      <c r="FG2" s="11" t="n"/>
+      <c r="FH2" s="11" t="n"/>
+      <c r="FI2" s="12" t="n"/>
       <c r="FJ2" s="2" t="inlineStr">
         <is>
           <t>HF Med - ARB</t>
         </is>
       </c>
-      <c r="FK2" s="2" t="n"/>
-      <c r="FL2" s="2" t="n"/>
-      <c r="FM2" s="2" t="n"/>
+      <c r="FK2" s="11" t="n"/>
+      <c r="FL2" s="11" t="n"/>
+      <c r="FM2" s="12" t="n"/>
       <c r="FN2" s="2" t="inlineStr">
         <is>
           <t>HF Med - Sacubitril–Valsartan</t>
         </is>
       </c>
-      <c r="FO2" s="2" t="n"/>
-      <c r="FP2" s="2" t="n"/>
-      <c r="FQ2" s="2" t="n"/>
+      <c r="FO2" s="11" t="n"/>
+      <c r="FP2" s="11" t="n"/>
+      <c r="FQ2" s="12" t="n"/>
       <c r="FR2" s="2" t="inlineStr">
         <is>
           <t>HF Med - Beta-Blocker</t>
         </is>
       </c>
-      <c r="FS2" s="2" t="n"/>
-      <c r="FT2" s="2" t="n"/>
-      <c r="FU2" s="2" t="n"/>
+      <c r="FS2" s="11" t="n"/>
+      <c r="FT2" s="11" t="n"/>
+      <c r="FU2" s="12" t="n"/>
       <c r="FV2" s="2" t="inlineStr">
         <is>
           <t>HF Med - Mineralocorticoid Receptor Antagonist</t>
         </is>
       </c>
-      <c r="FW2" s="2" t="n"/>
-      <c r="FX2" s="2" t="n"/>
-      <c r="FY2" s="2" t="n"/>
+      <c r="FW2" s="11" t="n"/>
+      <c r="FX2" s="11" t="n"/>
+      <c r="FY2" s="12" t="n"/>
       <c r="FZ2" s="2" t="inlineStr">
         <is>
           <t>HF Med - Digitalis</t>
         </is>
       </c>
-      <c r="GA2" s="2" t="n"/>
-      <c r="GB2" s="2" t="n"/>
-      <c r="GC2" s="2" t="n"/>
+      <c r="GA2" s="11" t="n"/>
+      <c r="GB2" s="11" t="n"/>
+      <c r="GC2" s="12" t="n"/>
       <c r="GD2" s="2" t="inlineStr">
         <is>
           <t>Primary Composite (Worsening HF or CV Death)</t>
         </is>
       </c>
-      <c r="GE2" s="2" t="n"/>
-      <c r="GF2" s="2" t="n"/>
-      <c r="GG2" s="2" t="n"/>
+      <c r="GE2" s="11" t="n"/>
+      <c r="GF2" s="11" t="n"/>
+      <c r="GG2" s="12" t="n"/>
       <c r="GH2" s="2" t="inlineStr">
         <is>
           <t>Hospitalization or Urgent HF Visit</t>
         </is>
       </c>
-      <c r="GI2" s="2" t="n"/>
-      <c r="GJ2" s="2" t="n"/>
-      <c r="GK2" s="2" t="n"/>
+      <c r="GI2" s="11" t="n"/>
+      <c r="GJ2" s="11" t="n"/>
+      <c r="GK2" s="12" t="n"/>
       <c r="GL2" s="2" t="inlineStr">
         <is>
           <t>Urgent Heart-Failure Visit</t>
         </is>
       </c>
-      <c r="GM2" s="2" t="n"/>
-      <c r="GN2" s="2" t="n"/>
-      <c r="GO2" s="2" t="n"/>
+      <c r="GM2" s="11" t="n"/>
+      <c r="GN2" s="11" t="n"/>
+      <c r="GO2" s="12" t="n"/>
       <c r="GP2" s="2" t="inlineStr">
         <is>
           <t>Cardiovascular Death</t>
         </is>
       </c>
-      <c r="GQ2" s="2" t="n"/>
-      <c r="GR2" s="2" t="n"/>
-      <c r="GS2" s="2" t="n"/>
+      <c r="GQ2" s="11" t="n"/>
+      <c r="GR2" s="11" t="n"/>
+      <c r="GS2" s="12" t="n"/>
       <c r="GT2" s="2" t="inlineStr">
         <is>
           <t>CV Death or HF Hospitalization</t>
         </is>
       </c>
-      <c r="GU2" s="2" t="n"/>
-      <c r="GV2" s="2" t="n"/>
-      <c r="GW2" s="2" t="n"/>
+      <c r="GU2" s="11" t="n"/>
+      <c r="GV2" s="11" t="n"/>
+      <c r="GW2" s="12" t="n"/>
       <c r="GX2" s="2" t="inlineStr">
         <is>
           <t>Total HF Hospitalizations and CV Deaths</t>
         </is>
       </c>
-      <c r="GY2" s="2" t="n"/>
-      <c r="GZ2" s="2" t="n"/>
-      <c r="HA2" s="2" t="n"/>
+      <c r="GY2" s="11" t="n"/>
+      <c r="GZ2" s="11" t="n"/>
+      <c r="HA2" s="12" t="n"/>
       <c r="HB2" s="2" t="inlineStr">
         <is>
           <t>Change in KCCQ Total Symptom Score</t>
         </is>
       </c>
-      <c r="HC2" s="2" t="n"/>
-      <c r="HD2" s="2" t="n"/>
-      <c r="HE2" s="2" t="n"/>
+      <c r="HC2" s="11" t="n"/>
+      <c r="HD2" s="11" t="n"/>
+      <c r="HE2" s="12" t="n"/>
       <c r="HF2" s="2" t="inlineStr">
         <is>
           <t>Worsening Renal Function Composite</t>
         </is>
       </c>
-      <c r="HG2" s="2" t="n"/>
-      <c r="HH2" s="2" t="n"/>
-      <c r="HI2" s="2" t="n"/>
+      <c r="HG2" s="11" t="n"/>
+      <c r="HH2" s="11" t="n"/>
+      <c r="HI2" s="12" t="n"/>
       <c r="HJ2" s="2" t="inlineStr">
         <is>
           <t>Death from Any Cause</t>
         </is>
       </c>
-      <c r="HK2" s="2" t="n"/>
-      <c r="HL2" s="2" t="n"/>
-      <c r="HM2" s="2" t="n"/>
+      <c r="HK2" s="11" t="n"/>
+      <c r="HL2" s="11" t="n"/>
+      <c r="HM2" s="12" t="n"/>
       <c r="HN2" s="2" t="inlineStr">
         <is>
           <t>Discontinuation Due to Adverse Event</t>
         </is>
       </c>
-      <c r="HO2" s="2" t="n"/>
-      <c r="HP2" s="2" t="n"/>
-      <c r="HQ2" s="2" t="n"/>
+      <c r="HO2" s="11" t="n"/>
+      <c r="HP2" s="11" t="n"/>
+      <c r="HQ2" s="12" t="n"/>
       <c r="HR2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Volume Depletion</t>
         </is>
       </c>
-      <c r="HS2" s="2" t="n"/>
-      <c r="HT2" s="2" t="n"/>
-      <c r="HU2" s="2" t="n"/>
+      <c r="HS2" s="11" t="n"/>
+      <c r="HT2" s="11" t="n"/>
+      <c r="HU2" s="12" t="n"/>
       <c r="HV2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Renal Adverse Event</t>
         </is>
       </c>
-      <c r="HW2" s="2" t="n"/>
-      <c r="HX2" s="2" t="n"/>
-      <c r="HY2" s="2" t="n"/>
+      <c r="HW2" s="11" t="n"/>
+      <c r="HX2" s="11" t="n"/>
+      <c r="HY2" s="12" t="n"/>
       <c r="HZ2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Fracture</t>
         </is>
       </c>
-      <c r="IA2" s="2" t="n"/>
-      <c r="IB2" s="2" t="n"/>
-      <c r="IC2" s="2" t="n"/>
+      <c r="IA2" s="11" t="n"/>
+      <c r="IB2" s="11" t="n"/>
+      <c r="IC2" s="12" t="n"/>
       <c r="ID2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Amputation</t>
         </is>
       </c>
-      <c r="IE2" s="2" t="n"/>
-      <c r="IF2" s="2" t="n"/>
-      <c r="IG2" s="2" t="n"/>
+      <c r="IE2" s="11" t="n"/>
+      <c r="IF2" s="11" t="n"/>
+      <c r="IG2" s="12" t="n"/>
       <c r="IH2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Major Hypoglycemia</t>
         </is>
       </c>
-      <c r="II2" s="2" t="n"/>
-      <c r="IJ2" s="2" t="n"/>
-      <c r="IK2" s="2" t="n"/>
+      <c r="II2" s="11" t="n"/>
+      <c r="IJ2" s="11" t="n"/>
+      <c r="IK2" s="12" t="n"/>
       <c r="IL2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Diabetic Ketoacidosis</t>
         </is>
       </c>
-      <c r="IM2" s="2" t="n"/>
-      <c r="IN2" s="2" t="n"/>
-      <c r="IO2" s="2" t="n"/>
+      <c r="IM2" s="11" t="n"/>
+      <c r="IN2" s="11" t="n"/>
+      <c r="IO2" s="12" t="n"/>
       <c r="IP2" s="2" t="inlineStr">
         <is>
           <t>Adverse Event - Fournier's Gangrene</t>
         </is>
       </c>
-      <c r="IQ2" s="2" t="n"/>
-      <c r="IR2" s="2" t="n"/>
-      <c r="IS2" s="2" t="n"/>
+      <c r="IQ2" s="11" t="n"/>
+      <c r="IR2" s="11" t="n"/>
+      <c r="IS2" s="12" t="n"/>
       <c r="IT2" s="2" t="inlineStr">
         <is>
           <t>Glycated Hemoglobin (HbA1c) Change</t>
         </is>
       </c>
-      <c r="IU2" s="2" t="n"/>
-      <c r="IV2" s="2" t="n"/>
-      <c r="IW2" s="2" t="n"/>
+      <c r="IU2" s="11" t="n"/>
+      <c r="IV2" s="11" t="n"/>
+      <c r="IW2" s="12" t="n"/>
       <c r="IX2" s="2" t="inlineStr">
         <is>
           <t>Serum Creatinine Change</t>
         </is>
       </c>
-      <c r="IY2" s="2" t="n"/>
-      <c r="IZ2" s="2" t="n"/>
-      <c r="JA2" s="2" t="n"/>
+      <c r="IY2" s="11" t="n"/>
+      <c r="IZ2" s="11" t="n"/>
+      <c r="JA2" s="12" t="n"/>
       <c r="JB2" s="2" t="inlineStr">
         <is>
           <t>Hematocrit Change</t>
         </is>
       </c>
-      <c r="JC2" s="2" t="n"/>
-      <c r="JD2" s="2" t="n"/>
-      <c r="JE2" s="2" t="n"/>
+      <c r="JC2" s="11" t="n"/>
+      <c r="JD2" s="11" t="n"/>
+      <c r="JE2" s="12" t="n"/>
       <c r="JF2" s="2" t="inlineStr">
         <is>
           <t>NT-proBNP Change</t>
         </is>
       </c>
-      <c r="JG2" s="2" t="n"/>
-      <c r="JH2" s="2" t="n"/>
-      <c r="JI2" s="2" t="n"/>
+      <c r="JG2" s="11" t="n"/>
+      <c r="JH2" s="11" t="n"/>
+      <c r="JI2" s="12" t="n"/>
       <c r="JJ2" s="2" t="inlineStr">
         <is>
           <t>Body Weight Change</t>
         </is>
       </c>
-      <c r="JK2" s="2" t="n"/>
-      <c r="JL2" s="2" t="n"/>
-      <c r="JM2" s="2" t="n"/>
+      <c r="JK2" s="11" t="n"/>
+      <c r="JL2" s="11" t="n"/>
+      <c r="JM2" s="12" t="n"/>
       <c r="JN2" s="2" t="inlineStr">
         <is>
           <t>Systolic Blood Pressure Change</t>
         </is>
       </c>
-      <c r="JO2" s="2" t="n"/>
-      <c r="JP2" s="2" t="n"/>
-      <c r="JQ2" s="2" t="n"/>
+      <c r="JO2" s="11" t="n"/>
+      <c r="JP2" s="11" t="n"/>
+      <c r="JQ2" s="12" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr"/>
@@ -10057,7 +10373,6 @@
     <mergeCell ref="GP2:GS2"/>
     <mergeCell ref="IH2:IK2"/>
     <mergeCell ref="FJ2:FM2"/>
-    <mergeCell ref="JJ2:JM2"/>
     <mergeCell ref="JB2:JE2"/>
     <mergeCell ref="AE2:AI2"/>
     <mergeCell ref="IT2:IW2"/>
@@ -10095,13 +10410,15 @@
     <mergeCell ref="IP2:IS2"/>
     <mergeCell ref="FR2:FU2"/>
     <mergeCell ref="HJ2:HM2"/>
+    <mergeCell ref="JJ2:JM2"/>
+    <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="IX2:JA2"/>
-    <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="CD2:CG2"/>
     <mergeCell ref="HV2:HY2"/>
     <mergeCell ref="BV2:BY2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10248,6 +10565,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10436,6 +10754,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11277,6 +11596,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -21311,6 +21631,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -26777,6 +27098,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -26843,6 +27165,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -35233,6 +35556,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -37043,5 +37367,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>